<commit_message>
Split tag generation into an explicit "clear data" step first
main.py now runs three visible stages instead of two: clear the raw
bulletin's data cells (keep only the year headers), THEN insert tags
into the cleared blank, THEN fill tags with fresh Excel data. Produces
a new intermediate artifact, output/Бюллетень_ОЧИЩЕННЫЙ.docx, so
anyone opening the file between stages sees a clean blank template --
no stale numbers from the prior period, no {{...}} placeholders either.

Implemented as a `clear_only` flag on generate_word_template rather
than a second copy of the matching logic: the same header/column
detection already used for tagging decides which cells to blank, so
"what gets cleared" and "what gets tagged" can never drift apart from
each other by construction.

Verified: identical result to the previous single-pass pipeline (0
lost/wrong tags vs. the prior known-good run) and a fresh whole-document
sweep finds 0 remaining raw numbers sitting next to tags.
</commit_message>
<xml_diff>
--- a/output/неиспользованные_показатели.xlsx
+++ b/output/неиспользованные_показатели.xlsx
@@ -488,11 +488,11 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.7</v>
+        <v>0.87</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>коэффициент обеспеченности собственными оборотными средствами 2023 401 9 846 2 40 7 111 1 704 2 14 6</t>
+          <t>коэффициент обеспеченности собственными оборотными средствами 2023</t>
         </is>
       </c>
     </row>
@@ -526,51 +526,51 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.6</v>
+        <v>0.87</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>коэффициент обеспеченности собственными оборотными средствами 2023 35 6 28 9 50 9 98 8 96 9 81 8 29 4 59 0 72 4 62 4 49 2 68 9 7 2</t>
+          <t>коэффициент обеспеченности собственными оборотными средствами 2023</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>230</v>
+        <v>112</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>T24_000000_t29Ved14.xlsx</t>
+          <t>T24_000000_t23Ved14mo8.xlsx</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>от переподажи финансовых вложений</t>
+          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) прочие расходы</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>OtPereprodFinVlozh</t>
+          <t>OtcGo(raSalProDohIRasProRas</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>0.52</v>
+        <v>0.67</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>в том числе от продажи внеоборотных активов кроме финансовых вложений 14 403 27 862</t>
+          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -579,32 +579,32 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) прочие расходы</t>
+          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) прочие доходы</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>OtcGo(raSalProDohIRasProRas</t>
+          <t>OtcGo(raSalProDohIRasProDoh</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>19</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>0.43</v>
+        <v>0.66</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов 26 192 421 24 539 666 16 212 8 936 1 515 800 669 10</t>
+          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -613,32 +613,32 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) прочие доходы</t>
+          <t>отчетный год отложенный налог на прибыль</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>OtcGo(raSalProDohIRasProDoh</t>
+          <t>OtcGoOtlNalNaPri_1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>0.42</v>
+        <v>0.59</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов 26 192 421 24 539 666 16 212 8 936 1 515 800 669 10</t>
+          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -647,66 +647,66 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) доходы от участия в других организациях</t>
+          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) проценты к уплате</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OtcGo(raSalProDohIRasDohOtUchVDruOrg</t>
+          <t>OtcGo(raSalProDohIRasProKUpl</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>0.39</v>
+        <v>0.59</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов 26 192 421 24 539 666 16 212 8 936 1 515 800 669 10</t>
+          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>109</v>
+        <v>230</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>T24_000000_t23Ved14mo8.xlsx</t>
+          <t>T24_000000_t29Ved14.xlsx</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) проценты к получению</t>
+          <t>от переподажи финансовых вложений</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OtcGo(raSalProDohIRasProKPol</t>
+          <t>OtPereprodFinVlozh</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>0.38</v>
+        <v>0.59</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов 26 192 421 24 539 666 16 212 8 936 1 515 800 669 10</t>
+          <t>в том числе от продажи внеоборотных активов кроме финансовых вложений</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -715,32 +715,32 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) проценты к уплате</t>
+          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) проценты к получению</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>OtcGo(raSalProDohIRasProKUpl</t>
+          <t>OtcGo(raSalProDohIRasProKPol</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>0.38</v>
+        <v>0.58</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов 26 192 421 24 539 666 16 212 8 936 1 515 800 669 10</t>
+          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -749,32 +749,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>отчетный год отложенный налог на прибыль</t>
+          <t>отчетный год (расшифровка сальдо прочих доходов и расходов) доходы от участия в других организациях</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>OtcGoOtlNalNaPri_1</t>
+          <t>OtcGo(raSalProDohIRasDohOtUchVDruOrg</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>0.36</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль 3 476 083 3 675 830 4 840 128 197 30 755 13 338 29 046 19 468 35 5</t>
+          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -783,66 +783,66 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>отчетный год налог на прибыль от операций, результат которых не включается в чистую прибыль (убыток) периода</t>
+          <t>отчетный год уровень коммерческих и управленческих расходов к валовой прибыли</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OtcGoNalNaPriOtOpeRezKotNeVklVChiPri(ubPer</t>
+          <t>OtcGoUroKomIUprRasKValPri</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>0.36</v>
+        <v>0.55</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль 3 476 083 3 675 830 4 840 128 197 30 755 13 338 29 046 19 468 35 5</t>
+          <t>коммерческие и управленческие расходы коммерческие и управленческие расходы</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>9</v>
+        <v>104</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>T24_000000_t01Ved14.xlsx</t>
+          <t>T24_000000_t23Ved14mo8.xlsx</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>валюта баланса убыточных организаций, на конец года в % к валюте баланса</t>
+          <t>отчетный год текущий налог на прибыль</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ValBalUbyOrgNaKonGoV%KValBal</t>
+          <t>OtcGoTekNalNaPri_1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>0.35</v>
+        <v>0.54</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>валюта баланса 2023 1 142 1 142 236 236 656 629 639 388 17 241</t>
+          <t>текущий налог на прибыль текущий налог на прибыль текущий налог на прибыль</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -851,100 +851,100 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>отчетный год текущий налог на прибыль</t>
+          <t>отчетный год сальдо прочих доходов и расходов</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>OtcGoTekNalNaPri_1</t>
+          <t>OtcGoSalProDohIRas_1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>0.33</v>
+        <v>0.53</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>текущий налог на прибыль текущий налог на прибыль текущий налог на прибыль 4 371 599 3 277 816 1 050 8 472 689 258 348 80 221 236 978 1 390 251 259</t>
+          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>T24_000000_t01Ved14.xlsx</t>
+          <t>T24_000000_t23Ved14mo8.xlsx</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>валюта баланса убыточных организаций, на конец года итог актива убыточных организаций</t>
+          <t>отчетный год прибыль (убыток) до налогообложения</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ValBalUbyOrgNaKonGoItAktUbyOrg</t>
+          <t>OtcGoPri(ubDoNal_1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>0.32</v>
+        <v>0.52</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>валюта баланса 2023 1 142 1 142 236 236 656 629 639 388 17 241</t>
+          <t>прибыль убыток до налогообложения прибыль убыток до налогообложения прибыль убыток до налогообложения</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>36</v>
+        <v>106</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>T24_000000_t13Ved14.xlsx</t>
+          <t>T24_000000_t23Ved14mo8.xlsx</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>средняя стоимость оборотных активов, тыс.рублей</t>
+          <t>отчетный год прочее</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SreStoOboAktTys</t>
+          <t>OtcGoPro_1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>0.32</v>
+        <v>0.51</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>запасы длительность 1 оборота 0 0 0 0 0 0 0 0 53 6 600 4 1 5</t>
+          <t>прочее прочее прочее</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -953,32 +953,32 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>отчетный год сальдо прочих доходов и расходов</t>
+          <t>отчетный год чистая прибыль (убыток) отчетного периода</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>OtcGoSalProDohIRas_1</t>
+          <t>OtcGoChiPri(ubOtcPer_1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>0.32</v>
+        <v>0.5</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>сальдо прочих доходов и расходов сальдо прочих доходов и расходов сальдо прочих доходов и расходов 26 192 421 24 539 666 16 212 8 936 1 515 800 669 10</t>
+          <t>на конец года тысяч рублей прибыль убыток от продаж прибыль убыток от продаж</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -987,80 +987,80 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>отчетный год уровень коммерческих и управленческих расходов к валовой прибыли</t>
+          <t>отчетный год налог на прибыль от операций, результат которых не включается в чистую прибыль (убыток) периода</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>OtcGoUroKomIUprRasKValPri</t>
+          <t>OtcGoNalNaPriOtOpeRezKotNeVklVChiPri(ubPer</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>24</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
-        <v>0.32</v>
+        <v>0.49</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">коммерческие и управленческие расходы коммерческие и управленческие расходы 50 117 067 34 775 932 59 731 12 931 2 008 4 451 768 1 899 638 1 619 509 3 </t>
+          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>103</v>
+        <v>36</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>T24_000000_t23Ved14mo8.xlsx</t>
+          <t>T24_000000_t13Ved14.xlsx</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>отчетный год прибыль (убыток) до налогообложения</t>
+          <t>средняя стоимость оборотных активов, тыс.рублей</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>OtcGoPri(ubDoNal_1</t>
+          <t>SreStoOboAktTys</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль 3 476 083 3 675 830 4 840 128 197 30 755 13 338 29 046 19 468 35 5</t>
+          <t>оборотные активы длительность 1 оборота</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>T24_000000_t23Ved14mo8.xlsx</t>
+          <t>T24_000000_t01Ved14.xlsx</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>отчетный год чистая прибыль (убыток) отчетного периода</t>
+          <t>валюта баланса убыточных организаций, на конец года в % к валюте баланса</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>OtcGoChiPri(ubOtcPer_1</t>
+          <t>ValBalUbyOrgNaKonGoV%KValBal</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1070,31 +1070,31 @@
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
-        <v>0.3</v>
+        <v>0.39</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль 3 476 083 3 675 830 4 840 128 197 30 755 13 338 29 046 19 468 35 5</t>
+          <t>валюта баланса 2023 валюта баланса 2023 валюта баланса 2023 валюта баланса 2023</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>106</v>
+        <v>8</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>T24_000000_t23Ved14mo8.xlsx</t>
+          <t>T24_000000_t01Ved14.xlsx</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>отчетный год прочее</t>
+          <t>валюта баланса убыточных организаций, на конец года итог актива убыточных организаций</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>OtcGoPro_1</t>
+          <t>ValBalUbyOrgNaKonGoItAktUbyOrg</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1104,17 +1104,17 @@
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
-        <v>0.24</v>
+        <v>0.38</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>продолжение таблицы 12</t>
+          <t>валюта баланса 2023 валюта баланса 2023 валюта баланса 2023 валюта баланса 2023</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1123,32 +1123,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>отчетный год совокупный финансовый результат периода</t>
+          <t>отчетный год результат от прочих операций, не включаемых в чистую прибыль (убыток) периода</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>OtcGoSovFinRezPer_1</t>
+          <t>OtcGoRezOtProOpeNeVklVChiPri(ubPer_1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
-        <v>0.24</v>
+        <v>0.38</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль 3 476 083 3 675 830 4 840 128 197 30 755 13 338 29 046 19 468 35 5</t>
+          <t>на конец года тысяч рублей прибыль убыток от продаж прибыль убыток от продаж</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1157,32 +1157,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>отчетный год результат от прочих операций, не включаемых в чистую прибыль (убыток) периода</t>
+          <t>отчетный год совокупный финансовый результат периода</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>OtcGoRezOtProOpeNeVklVChiPri(ubPer_1</t>
+          <t>OtcGoSovFinRezPer_1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
-        <v>0.23</v>
+        <v>0.36</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>текущий налог на прибыль текущий налог на прибыль текущий налог на прибыль 4 371 599 3 277 816 1 050 8 472 689 258 348 80 221 236 978 1 390 251 259</t>
+          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1191,94 +1191,94 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>валюта баланса убыточных организаций, на конец года в % к валюте баланса</t>
+          <t>валюта баланса убыточных организаций, на конец года итог актива убыточных организаций</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ValBalUbyOrgNaKonGoV%KValBal_1</t>
+          <t>ValBalUbyOrgNaKonGoItAktUbyOrg_1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="n">
-        <v>0.21</v>
+        <v>0.35</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>валюта баланса 2023 731 078 261 510 134 382 473 989 147 908 3 826 98 918 91 189 798 59 137 171 25 203 480 44 161 896 7 803 414 40 126 683 821 732</t>
+          <t>на конец года тысяч рублей оборотные активы 2023</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>113</v>
+        <v>17</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>T24_000000_t23Ved14mo8.xlsx</t>
+          <t>T24_000000_t01Ved14mo8.xlsx</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>отчетный год результат от переоценки внеоборотных активов, не включаемых в чистую прибыль (убыток) периода</t>
+          <t>валюта баланса убыточных организаций, на конец года в % к валюте баланса</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>OtcGoRezOtPerVneAktNeVklVChiPri(ubPer_1</t>
+          <t>ValBalUbyOrgNaKonGoV%KValBal_1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
-        <v>0.21</v>
+        <v>0.34</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>отложенный налог на прибыль отложенный налог на прибыль отложенный налог на прибыль 3 476 083 3 675 830 4 840 128 197 30 755 13 338 29 046 19 468 35 5</t>
+          <t>на конец года тысяч рублей оборотные активы 2023</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>16</v>
+        <v>113</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>T24_000000_t01Ved14mo8.xlsx</t>
+          <t>T24_000000_t23Ved14mo8.xlsx</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>валюта баланса убыточных организаций, на конец года итог актива убыточных организаций</t>
+          <t>отчетный год результат от переоценки внеоборотных активов, не включаемых в чистую прибыль (убыток) периода</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ValBalUbyOrgNaKonGoItAktUbyOrg_1</t>
+          <t>OtcGoRezOtPerVneAktNeVklVChiPri(ubPer_1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="n">
-        <v>0.2</v>
+        <v>0.34</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>валюта баланса 2023 731 078 261 510 134 382 473 989 147 908 3 826 98 918 91 189 798 59 137 171 25 203 480 44 161 896 7 803 414 40 126 683 821 732</t>
+          <t>на конец года тысяч рублей прибыль убыток от продаж прибыль убыток от продаж</t>
         </is>
       </c>
     </row>

</xml_diff>